<commit_message>
problem with lecton's 5 task whith iris dataset
</commit_message>
<xml_diff>
--- a/lesson3/answer1.xlsx
+++ b/lesson3/answer1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\python\data_science_camp\lesson3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49BB2E11-4807-4BE0-99A6-E3DBD9D74CC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F080D2A1-C84F-4FCC-9850-5C998BCA0E11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="108" yWindow="1836" windowWidth="12108" windowHeight="9420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="3924" yWindow="5268" windowWidth="17400" windowHeight="7164" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -496,6 +496,7 @@
   <dimension ref="A1:V16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="1" max="1" width="16.21875" customWidth="1"/>
     <col min="3" max="3" width="17.33203125" customWidth="1"/>
     <col min="4" max="4" width="18.33203125" customWidth="1"/>
     <col min="5" max="5" width="14.5546875" customWidth="1"/>

</xml_diff>